<commit_message>
One frozen canonical framework contract
</commit_message>
<xml_diff>
--- a/src/Thesis_ML/assets/templates/thesis_experiment_program.xlsx
+++ b/src/Thesis_ML/assets/templates/thesis_experiment_program.xlsx
@@ -1814,6 +1814,18 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>thesis_protocol_schema_version</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>thesis-protocol-v1</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>

</xml_diff>